<commit_message>
update analysed files containing the full linear video results
</commit_message>
<xml_diff>
--- a/Analysed/GPT/Analysis_Summary_Depth_without_vernier_gpt5.3Instant.xlsx
+++ b/Analysed/GPT/Analysis_Summary_Depth_without_vernier_gpt5.3Instant.xlsx
@@ -449,7 +449,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5.4635 ± nan</t>
+          <t>4.8622 ± 4.7876</t>
         </is>
       </c>
     </row>
@@ -461,7 +461,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>5.6826 ± nan</t>
+          <t>5.3004 ± 5.0113</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.8125 ± nan</t>
+          <t>0.5968 ± 0.2669</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,20 +521,96 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>V2_10 divisions_per_second</t>
+          <t>V2_0.5 divisions_per_second</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>132</v>
+      </c>
+      <c r="C2" t="n">
+        <v>4.300681818181817</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5.430714766841274</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.2900763358778626</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>V3_0.8 divisions_per_second</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>83</v>
+      </c>
+      <c r="C3" t="n">
+        <v>9.499638554216867</v>
+      </c>
+      <c r="D3" t="n">
+        <v>9.874604826621049</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.7439024390243902</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>V4_1.7 divisions_per_second</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>58</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.2412068965517241</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.2804399253389893</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.7368421052631579</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>V5_2.5 divisions_per_second</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>51</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.2174509803921567</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.2494189325644079</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>V7_10 divisions_per_second</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>49</v>
       </c>
-      <c r="C2" t="n">
-        <v>5.463469387755102</v>
-      </c>
-      <c r="D2" t="n">
-        <v>5.682601624651317</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.8125</v>
+      <c r="C6" t="n">
+        <v>10.05204081632653</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10.66704107548679</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.3333333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>